<commit_message>
Finalized MCU pin assignment. Added STM32L476 datasheet.
</commit_message>
<xml_diff>
--- a/hardware/schematics/pin_map.xlsx
+++ b/hardware/schematics/pin_map.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95715795-A8E8-49A2-899D-8EE63D5E1D5D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DCBCBC4-3C8F-4469-B33E-B4DADDE24829}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="96">
   <si>
     <t>Function</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Debug UART</t>
   </si>
   <si>
-    <t>UART_TX</t>
-  </si>
-  <si>
     <t>Peripheral</t>
   </si>
   <si>
@@ -46,9 +43,6 @@
     <t>Signal</t>
   </si>
   <si>
-    <t>UART_RX</t>
-  </si>
-  <si>
     <t>GPS UART</t>
   </si>
   <si>
@@ -242,6 +236,78 @@
   </si>
   <si>
     <t>AF14</t>
+  </si>
+  <si>
+    <t>Power ack</t>
+  </si>
+  <si>
+    <t>Analog input 1</t>
+  </si>
+  <si>
+    <t>Analog input 2</t>
+  </si>
+  <si>
+    <t>ADC1</t>
+  </si>
+  <si>
+    <t>ADC1_IN3</t>
+  </si>
+  <si>
+    <t>ADC1_IN4</t>
+  </si>
+  <si>
+    <t>PC2</t>
+  </si>
+  <si>
+    <t>PC3</t>
+  </si>
+  <si>
+    <t>ANA</t>
+  </si>
+  <si>
+    <t>PB9</t>
+  </si>
+  <si>
+    <t>PB8</t>
+  </si>
+  <si>
+    <t>UART extension</t>
+  </si>
+  <si>
+    <t>USART1</t>
+  </si>
+  <si>
+    <t>USART3_RX</t>
+  </si>
+  <si>
+    <t>USART3_TX</t>
+  </si>
+  <si>
+    <t>USART1_RX</t>
+  </si>
+  <si>
+    <t>USART1_TX</t>
+  </si>
+  <si>
+    <t>LPUART1_RX</t>
+  </si>
+  <si>
+    <t>LPUART1_TX</t>
+  </si>
+  <si>
+    <t>PC8</t>
+  </si>
+  <si>
+    <t>PC6</t>
+  </si>
+  <si>
+    <t>PC7</t>
+  </si>
+  <si>
+    <t>PC5</t>
+  </si>
+  <si>
+    <t>PC4</t>
   </si>
 </sst>
 </file>
@@ -941,7 +1007,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="24" style="11" customWidth="1"/>
@@ -954,10 +1020,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -968,32 +1034,32 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1001,428 +1067,482 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>8</v>
+        <v>87</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7" t="s">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7" t="s">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="12"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="12"/>
       <c r="B12" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
       <c r="B13" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="12"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="12"/>
       <c r="B17" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
       <c r="B18" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
       <c r="B19" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="D20" s="4" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D22" s="15"/>
+        <v>24</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>94</v>
+      </c>
       <c r="E22" s="16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="15"/>
+        <v>24</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>95</v>
+      </c>
       <c r="E23" s="16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D24" s="15"/>
+        <v>24</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>93</v>
+      </c>
       <c r="E24" s="16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C25" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="22" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="B27" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="D27" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="17"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="D28" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="6"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E31" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D33" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="17"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18" t="s">
+      <c r="E33" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D27" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="E27" s="19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="6"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="B29" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="C29" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="D29" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="E29" s="25" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
+      <c r="E34" s="8" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
+      <c r="A35" s="9"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
@@ -1459,6 +1579,13 @@
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
     </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated pin asignment with MCO pin. Deleted old accelerometer datasheet. Changing barometric sensor reference to MS5607.
</commit_message>
<xml_diff>
--- a/hardware/schematics/pin_map.xlsx
+++ b/hardware/schematics/pin_map.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DCBCBC4-3C8F-4469-B33E-B4DADDE24829}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203AC436-DF06-4F9D-B934-1F863DFB2216}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="100">
   <si>
     <t>Function</t>
   </si>
@@ -308,6 +308,18 @@
   </si>
   <si>
     <t>PC4</t>
+  </si>
+  <si>
+    <t>MCO</t>
+  </si>
+  <si>
+    <t>MCU_MCO</t>
+  </si>
+  <si>
+    <t>PA8</t>
+  </si>
+  <si>
+    <t>µC Clock Output</t>
   </si>
 </sst>
 </file>
@@ -1007,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="24" style="11" customWidth="1"/>
@@ -1062,93 +1074,97 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7" t="s">
+    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E6" s="8" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7" t="s">
+    <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="5" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1156,10 +1172,10 @@
       <c r="A10" s="12"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>58</v>
@@ -1167,17 +1183,15 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
-      <c r="B11" s="10" t="s">
-        <v>15</v>
-      </c>
+      <c r="B11" s="10"/>
       <c r="C11" s="10" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1186,57 +1200,59 @@
         <v>15</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6"/>
-      <c r="B13" s="7" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="12"/>
+      <c r="B13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6"/>
+      <c r="B14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E14" s="8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="5" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1244,10 +1260,10 @@
       <c r="A16" s="12"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>58</v>
@@ -1255,17 +1271,15 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="12"/>
-      <c r="B17" s="10" t="s">
-        <v>15</v>
-      </c>
+      <c r="B17" s="10"/>
       <c r="C17" s="10" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1274,80 +1288,78 @@
         <v>15</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E18" s="13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="6"/>
-      <c r="B19" s="7" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="12"/>
+      <c r="B19" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6"/>
+      <c r="B20" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E20" s="8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="6"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7" t="s">
+    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="6"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D22" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E22" s="8" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>15</v>
@@ -1356,7 +1368,7 @@
         <v>24</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E23" s="16" t="s">
         <v>24</v>
@@ -1364,7 +1376,7 @@
     </row>
     <row r="24" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>15</v>
@@ -1373,183 +1385,193 @@
         <v>24</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E24" s="16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B26" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C26" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="D26" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="E25" s="22" t="s">
+      <c r="E26" s="22" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
+    <row r="27" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B27" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C27" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D27" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="E26" s="16" t="s">
+      <c r="E27" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B28" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C28" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D28" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="17"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="17"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D29" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E29" s="19" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="6"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7" t="s">
+    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="6"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D30" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="E30" s="8" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="23" t="s">
+    <row r="31" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B31" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="C30" s="24" t="s">
+      <c r="C31" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="D30" s="24" t="s">
+      <c r="D31" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="E30" s="25" t="s">
+      <c r="E31" s="25" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E31" s="16" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>75</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E32" s="16" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E33" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B34" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C34" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E33" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7" t="s">
+    <row r="35" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="6"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D35" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E35" s="8" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-    </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
+      <c r="A36" s="9"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
@@ -1586,6 +1608,13 @@
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
     </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>